<commit_message>
Fix harmonized_data_schema typos with race6
</commit_message>
<xml_diff>
--- a/Resources/Admin/Crosswalks and Schemas.xlsx
+++ b/Resources/Admin/Crosswalks and Schemas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SHDTJB\Documents\LocalSave\Code\R\GitHub\WA-DOH-CHS-Death-Files-ETL\Resources\Admin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DA9971D-67F4-49C8-965B-6ED0067B6BFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAB0C845-FD16-4D9A-B0AF-26352C9E6F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5692" uniqueCount="731">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5693" uniqueCount="731">
   <si>
     <t>to_name</t>
   </si>
@@ -20284,6 +20284,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D60DD1-DC0B-4658-A996-7DC0B41964ED}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:H372"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -20319,7 +20320,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>4</v>
       </c>
@@ -20332,7 +20333,7 @@
       <c r="F2" s="20"/>
       <c r="G2" s="18"/>
     </row>
-    <row r="3" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
         <v>676</v>
       </c>
@@ -20353,7 +20354,7 @@
       </c>
       <c r="G3" s="18"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
         <v>676</v>
       </c>
@@ -20373,7 +20374,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
         <v>676</v>
       </c>
@@ -20393,7 +20394,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
         <v>676</v>
       </c>
@@ -20413,7 +20414,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
         <v>676</v>
       </c>
@@ -20433,7 +20434,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
         <v>676</v>
       </c>
@@ -20453,7 +20454,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
         <v>682</v>
       </c>
@@ -20474,7 +20475,7 @@
       </c>
       <c r="G9" s="18"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
         <v>682</v>
       </c>
@@ -20494,7 +20495,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
         <v>682</v>
       </c>
@@ -20514,7 +20515,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
         <v>682</v>
       </c>
@@ -20534,7 +20535,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
         <v>682</v>
       </c>
@@ -20554,7 +20555,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
         <v>682</v>
       </c>
@@ -20574,7 +20575,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
         <v>682</v>
       </c>
@@ -20594,7 +20595,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
         <v>682</v>
       </c>
@@ -20614,7 +20615,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
         <v>682</v>
       </c>
@@ -20634,7 +20635,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
         <v>682</v>
       </c>
@@ -20654,7 +20655,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
         <v>682</v>
       </c>
@@ -20674,7 +20675,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
         <v>692</v>
       </c>
@@ -20695,7 +20696,7 @@
       </c>
       <c r="G20" s="18"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
         <v>692</v>
       </c>
@@ -20715,7 +20716,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
         <v>692</v>
       </c>
@@ -20735,7 +20736,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
         <v>692</v>
       </c>
@@ -20755,7 +20756,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
         <v>692</v>
       </c>
@@ -20775,7 +20776,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
         <v>692</v>
       </c>
@@ -20795,7 +20796,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
         <v>692</v>
       </c>
@@ -20815,7 +20816,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
         <v>692</v>
       </c>
@@ -20835,7 +20836,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
         <v>692</v>
       </c>
@@ -20855,7 +20856,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
         <v>692</v>
       </c>
@@ -20875,7 +20876,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
         <v>692</v>
       </c>
@@ -20895,7 +20896,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
         <v>692</v>
       </c>
@@ -20915,7 +20916,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
         <v>692</v>
       </c>
@@ -20935,7 +20936,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
         <v>692</v>
       </c>
@@ -20955,7 +20956,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
         <v>692</v>
       </c>
@@ -20975,7 +20976,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
         <v>692</v>
       </c>
@@ -20995,7 +20996,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="12" t="s">
         <v>692</v>
       </c>
@@ -21015,7 +21016,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
         <v>692</v>
       </c>
@@ -21035,7 +21036,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="12" t="s">
         <v>692</v>
       </c>
@@ -21055,7 +21056,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
         <v>692</v>
       </c>
@@ -21075,7 +21076,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="40" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="17" t="s">
         <v>710</v>
       </c>
@@ -21096,7 +21097,7 @@
       </c>
       <c r="G40" s="18"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="12" t="s">
         <v>710</v>
       </c>
@@ -21116,7 +21117,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="12" t="s">
         <v>710</v>
       </c>
@@ -21136,7 +21137,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="12" t="s">
         <v>710</v>
       </c>
@@ -21156,7 +21157,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="12" t="s">
         <v>710</v>
       </c>
@@ -21176,7 +21177,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="12" t="s">
         <v>710</v>
       </c>
@@ -21196,7 +21197,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="12" t="s">
         <v>710</v>
       </c>
@@ -21216,7 +21217,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="12" t="s">
         <v>710</v>
       </c>
@@ -21236,7 +21237,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="12" t="s">
         <v>710</v>
       </c>
@@ -21256,7 +21257,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="12" t="s">
         <v>710</v>
       </c>
@@ -21276,7 +21277,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="12" t="s">
         <v>710</v>
       </c>
@@ -21296,7 +21297,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="12" t="s">
         <v>710</v>
       </c>
@@ -21316,7 +21317,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="12" t="s">
         <v>710</v>
       </c>
@@ -21336,7 +21337,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
         <v>710</v>
       </c>
@@ -21356,7 +21357,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="12" t="s">
         <v>710</v>
       </c>
@@ -21376,7 +21377,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="12" t="s">
         <v>710</v>
       </c>
@@ -21396,7 +21397,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="12" t="s">
         <v>710</v>
       </c>
@@ -21416,7 +21417,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="12" t="s">
         <v>710</v>
       </c>
@@ -21436,7 +21437,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="58" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="17" t="s">
         <v>6</v>
       </c>
@@ -21455,7 +21456,7 @@
       <c r="F58" s="20"/>
       <c r="G58" s="18"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="12" t="s">
         <v>6</v>
       </c>
@@ -21472,7 +21473,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="12" t="s">
         <v>6</v>
       </c>
@@ -21489,7 +21490,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="12" t="s">
         <v>6</v>
       </c>
@@ -21506,7 +21507,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="12" t="s">
         <v>6</v>
       </c>
@@ -21523,7 +21524,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="12" t="s">
         <v>6</v>
       </c>
@@ -21540,7 +21541,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="64" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="17" t="s">
         <v>7</v>
       </c>
@@ -21553,7 +21554,7 @@
       <c r="F64" s="20"/>
       <c r="G64" s="18"/>
     </row>
-    <row r="65" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="17" t="s">
         <v>523</v>
       </c>
@@ -21566,7 +21567,7 @@
       <c r="F65" s="20"/>
       <c r="G65" s="18"/>
     </row>
-    <row r="66" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="17" t="s">
         <v>9</v>
       </c>
@@ -21585,7 +21586,7 @@
       <c r="F66" s="20"/>
       <c r="G66" s="18"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="12" t="s">
         <v>9</v>
       </c>
@@ -21602,7 +21603,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="12" t="s">
         <v>9</v>
       </c>
@@ -21619,7 +21620,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="69" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="17" t="s">
         <v>10</v>
       </c>
@@ -21638,7 +21639,7 @@
       <c r="F69" s="20"/>
       <c r="G69" s="18"/>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="12" t="s">
         <v>10</v>
       </c>
@@ -21655,7 +21656,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="12" t="s">
         <v>10</v>
       </c>
@@ -21672,7 +21673,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="72" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="17" t="s">
         <v>12</v>
       </c>
@@ -21689,7 +21690,7 @@
       <c r="F72" s="20"/>
       <c r="G72" s="18"/>
     </row>
-    <row r="73" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="17" t="s">
         <v>14</v>
       </c>
@@ -21706,7 +21707,7 @@
       <c r="F73" s="20"/>
       <c r="G73" s="18"/>
     </row>
-    <row r="74" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="19" t="s">
         <v>16</v>
       </c>
@@ -21725,7 +21726,7 @@
       <c r="F74" s="20"/>
       <c r="G74" s="18"/>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="4" t="s">
         <v>16</v>
       </c>
@@ -21742,7 +21743,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
         <v>16</v>
       </c>
@@ -21759,7 +21760,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="4" t="s">
         <v>16</v>
       </c>
@@ -21776,7 +21777,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
         <v>16</v>
       </c>
@@ -21793,7 +21794,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="4" t="s">
         <v>16</v>
       </c>
@@ -21810,7 +21811,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
         <v>16</v>
       </c>
@@ -21827,7 +21828,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="4" t="s">
         <v>16</v>
       </c>
@@ -21844,7 +21845,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
         <v>16</v>
       </c>
@@ -21861,7 +21862,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="83" spans="1:8" s="19" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:8" s="19" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="34" t="s">
         <v>629</v>
       </c>
@@ -21874,7 +21875,7 @@
       <c r="F83" s="35"/>
       <c r="G83" s="17"/>
     </row>
-    <row r="84" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="34" t="s">
         <v>630</v>
       </c>
@@ -21887,7 +21888,7 @@
       <c r="F84" s="20"/>
       <c r="G84" s="18"/>
     </row>
-    <row r="85" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:8" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="34" t="s">
         <v>631</v>
       </c>
@@ -21900,7 +21901,7 @@
       <c r="F85" s="20"/>
       <c r="G85" s="18"/>
     </row>
-    <row r="86" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="34" t="s">
         <v>632</v>
       </c>
@@ -21913,7 +21914,7 @@
       <c r="F86" s="20"/>
       <c r="G86" s="18"/>
     </row>
-    <row r="87" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="34" t="s">
         <v>633</v>
       </c>
@@ -21926,7 +21927,7 @@
       <c r="F87" s="20"/>
       <c r="G87" s="18"/>
     </row>
-    <row r="88" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="17" t="s">
         <v>525</v>
       </c>
@@ -21940,7 +21941,7 @@
       <c r="G88" s="18"/>
       <c r="H88" s="18"/>
     </row>
-    <row r="89" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="17" t="s">
         <v>18</v>
       </c>
@@ -21953,7 +21954,7 @@
       <c r="F89" s="20"/>
       <c r="G89" s="18"/>
     </row>
-    <row r="90" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="17" t="s">
         <v>20</v>
       </c>
@@ -21966,7 +21967,7 @@
       <c r="F90" s="20"/>
       <c r="G90" s="18"/>
     </row>
-    <row r="91" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="17" t="s">
         <v>22</v>
       </c>
@@ -21985,7 +21986,7 @@
       <c r="F91" s="20"/>
       <c r="G91" s="18"/>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="12" t="s">
         <v>22</v>
       </c>
@@ -22002,7 +22003,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="12" t="s">
         <v>22</v>
       </c>
@@ -22019,7 +22020,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="12" t="s">
         <v>22</v>
       </c>
@@ -22036,7 +22037,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="12" t="s">
         <v>22</v>
       </c>
@@ -22053,7 +22054,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="12" t="s">
         <v>22</v>
       </c>
@@ -22070,7 +22071,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="12" t="s">
         <v>22</v>
       </c>
@@ -22087,7 +22088,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="98" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="17" t="s">
         <v>24</v>
       </c>
@@ -22100,7 +22101,7 @@
       <c r="F98" s="20"/>
       <c r="G98" s="18"/>
     </row>
-    <row r="99" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="17" t="s">
         <v>26</v>
       </c>
@@ -22113,7 +22114,7 @@
       <c r="F99" s="20"/>
       <c r="G99" s="18"/>
     </row>
-    <row r="100" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="17" t="s">
         <v>27</v>
       </c>
@@ -22126,7 +22127,7 @@
       <c r="F100" s="20"/>
       <c r="G100" s="18"/>
     </row>
-    <row r="101" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="17" t="s">
         <v>28</v>
       </c>
@@ -22139,7 +22140,7 @@
       <c r="F101" s="20"/>
       <c r="G101" s="18"/>
     </row>
-    <row r="102" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="17" t="s">
         <v>30</v>
       </c>
@@ -22152,7 +22153,7 @@
       <c r="F102" s="20"/>
       <c r="G102" s="18"/>
     </row>
-    <row r="103" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="17" t="s">
         <v>32</v>
       </c>
@@ -22165,7 +22166,7 @@
       <c r="F103" s="20"/>
       <c r="G103" s="18"/>
     </row>
-    <row r="104" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="17" t="s">
         <v>34</v>
       </c>
@@ -22178,7 +22179,7 @@
       <c r="F104" s="20"/>
       <c r="G104" s="18"/>
     </row>
-    <row r="105" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="17" t="s">
         <v>36</v>
       </c>
@@ -22191,7 +22192,7 @@
       <c r="F105" s="20"/>
       <c r="G105" s="18"/>
     </row>
-    <row r="106" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" s="17" t="s">
         <v>38</v>
       </c>
@@ -22204,7 +22205,7 @@
       <c r="F106" s="20"/>
       <c r="G106" s="18"/>
     </row>
-    <row r="107" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="17" t="s">
         <v>40</v>
       </c>
@@ -22223,7 +22224,7 @@
       <c r="F107" s="20"/>
       <c r="G107" s="18"/>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="12" t="s">
         <v>40</v>
       </c>
@@ -22240,7 +22241,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="12" t="s">
         <v>40</v>
       </c>
@@ -22257,7 +22258,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="12" t="s">
         <v>40</v>
       </c>
@@ -22274,7 +22275,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="12" t="s">
         <v>40</v>
       </c>
@@ -22291,7 +22292,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" s="12" t="s">
         <v>40</v>
       </c>
@@ -22308,7 +22309,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" s="12" t="s">
         <v>40</v>
       </c>
@@ -22325,7 +22326,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" s="12" t="s">
         <v>40</v>
       </c>
@@ -22342,7 +22343,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="115" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="17" t="s">
         <v>42</v>
       </c>
@@ -22355,7 +22356,7 @@
       <c r="F115" s="20"/>
       <c r="G115" s="18"/>
     </row>
-    <row r="116" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" s="17" t="s">
         <v>44</v>
       </c>
@@ -22376,7 +22377,7 @@
       </c>
       <c r="G116" s="18"/>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="12" t="s">
         <v>44</v>
       </c>
@@ -22396,7 +22397,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="12" t="s">
         <v>44</v>
       </c>
@@ -22416,7 +22417,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="12" t="s">
         <v>44</v>
       </c>
@@ -22436,7 +22437,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="12" t="s">
         <v>44</v>
       </c>
@@ -22456,7 +22457,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="12" t="s">
         <v>44</v>
       </c>
@@ -22476,7 +22477,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" s="12" t="s">
         <v>44</v>
       </c>
@@ -22496,7 +22497,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="12" t="s">
         <v>44</v>
       </c>
@@ -22516,7 +22517,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" s="12" t="s">
         <v>44</v>
       </c>
@@ -22536,7 +22537,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="125" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" s="17" t="s">
         <v>46</v>
       </c>
@@ -22557,7 +22558,7 @@
       </c>
       <c r="G125" s="18"/>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" s="12" t="s">
         <v>46</v>
       </c>
@@ -22577,7 +22578,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" s="12" t="s">
         <v>46</v>
       </c>
@@ -22597,7 +22598,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" s="12" t="s">
         <v>46</v>
       </c>
@@ -22617,7 +22618,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" s="12" t="s">
         <v>46</v>
       </c>
@@ -22637,7 +22638,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" s="12" t="s">
         <v>46</v>
       </c>
@@ -22657,7 +22658,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="12" t="s">
         <v>46</v>
       </c>
@@ -22677,7 +22678,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" s="12" t="s">
         <v>46</v>
       </c>
@@ -22697,7 +22698,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" s="12" t="s">
         <v>46</v>
       </c>
@@ -22717,7 +22718,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" s="12" t="s">
         <v>46</v>
       </c>
@@ -22737,7 +22738,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="135" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" s="19" t="s">
         <v>391</v>
       </c>
@@ -22750,7 +22751,7 @@
       <c r="F135" s="20"/>
       <c r="G135" s="18"/>
     </row>
-    <row r="136" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" s="19" t="s">
         <v>713</v>
       </c>
@@ -22763,7 +22764,7 @@
       <c r="F136" s="20"/>
       <c r="G136" s="18"/>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" s="4" t="s">
         <v>713</v>
       </c>
@@ -22771,7 +22772,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="138" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" s="17" t="s">
         <v>48</v>
       </c>
@@ -22790,7 +22791,7 @@
       <c r="F138" s="20"/>
       <c r="G138" s="18"/>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="12" t="s">
         <v>48</v>
       </c>
@@ -22807,7 +22808,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" s="12" t="s">
         <v>48</v>
       </c>
@@ -22824,7 +22825,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="141" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" s="17" t="s">
         <v>50</v>
       </c>
@@ -22843,7 +22844,7 @@
       <c r="F141" s="20"/>
       <c r="G141" s="18"/>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" s="12" t="s">
         <v>50</v>
       </c>
@@ -22860,7 +22861,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" s="12" t="s">
         <v>50</v>
       </c>
@@ -22877,7 +22878,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="144" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" s="17" t="s">
         <v>52</v>
       </c>
@@ -22896,7 +22897,7 @@
       <c r="F144" s="20"/>
       <c r="G144" s="18"/>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" s="12" t="s">
         <v>52</v>
       </c>
@@ -22913,7 +22914,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" s="12" t="s">
         <v>52</v>
       </c>
@@ -22930,7 +22931,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" s="12" t="s">
         <v>52</v>
       </c>
@@ -22947,7 +22948,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" s="12" t="s">
         <v>52</v>
       </c>
@@ -22964,7 +22965,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" s="12" t="s">
         <v>52</v>
       </c>
@@ -22981,7 +22982,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" s="12" t="s">
         <v>52</v>
       </c>
@@ -22998,7 +22999,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="151" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" s="17" t="s">
         <v>54</v>
       </c>
@@ -23017,7 +23018,7 @@
       <c r="F151" s="20"/>
       <c r="G151" s="18"/>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" s="12" t="s">
         <v>54</v>
       </c>
@@ -23034,7 +23035,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" s="12" t="s">
         <v>54</v>
       </c>
@@ -23051,7 +23052,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="154" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="17" t="s">
         <v>56</v>
       </c>
@@ -23070,7 +23071,7 @@
       <c r="F154" s="20"/>
       <c r="G154" s="18"/>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" s="12" t="s">
         <v>56</v>
       </c>
@@ -23087,7 +23088,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" s="12" t="s">
         <v>56</v>
       </c>
@@ -23104,7 +23105,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="157" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="17" t="s">
         <v>58</v>
       </c>
@@ -23123,7 +23124,7 @@
       <c r="F157" s="20"/>
       <c r="G157" s="18"/>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" s="12" t="s">
         <v>58</v>
       </c>
@@ -23140,7 +23141,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" s="12" t="s">
         <v>58</v>
       </c>
@@ -23157,7 +23158,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="160" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" s="17" t="s">
         <v>60</v>
       </c>
@@ -23170,7 +23171,7 @@
       <c r="F160" s="20"/>
       <c r="G160" s="18"/>
     </row>
-    <row r="161" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" s="17" t="s">
         <v>62</v>
       </c>
@@ -23183,7 +23184,7 @@
       <c r="F161" s="20"/>
       <c r="G161" s="18"/>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" s="12" t="s">
         <v>64</v>
       </c>
@@ -23200,7 +23201,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" s="12" t="s">
         <v>64</v>
       </c>
@@ -23217,7 +23218,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" s="12" t="s">
         <v>64</v>
       </c>
@@ -23234,7 +23235,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" s="12" t="s">
         <v>64</v>
       </c>
@@ -23251,7 +23252,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" s="12" t="s">
         <v>64</v>
       </c>
@@ -23268,7 +23269,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" s="12" t="s">
         <v>64</v>
       </c>
@@ -23285,7 +23286,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" s="12" t="s">
         <v>64</v>
       </c>
@@ -23302,7 +23303,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" s="12" t="s">
         <v>64</v>
       </c>
@@ -23319,7 +23320,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" s="12" t="s">
         <v>64</v>
       </c>
@@ -23336,7 +23337,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171" s="12" t="s">
         <v>64</v>
       </c>
@@ -23353,7 +23354,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="172" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A172" s="17" t="s">
         <v>66</v>
       </c>
@@ -23372,7 +23373,7 @@
       <c r="F172" s="20"/>
       <c r="G172" s="18"/>
     </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173" s="12" t="s">
         <v>66</v>
       </c>
@@ -23389,7 +23390,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174" s="12" t="s">
         <v>66</v>
       </c>
@@ -23406,7 +23407,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175" s="12" t="s">
         <v>67</v>
       </c>
@@ -23414,7 +23415,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="176" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176" s="17" t="s">
         <v>68</v>
       </c>
@@ -23427,7 +23428,7 @@
       <c r="F176" s="20"/>
       <c r="G176" s="18"/>
     </row>
-    <row r="177" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" s="17" t="s">
         <v>69</v>
       </c>
@@ -23440,7 +23441,7 @@
       <c r="F177" s="20"/>
       <c r="G177" s="18"/>
     </row>
-    <row r="178" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178" s="17" t="s">
         <v>71</v>
       </c>
@@ -23453,7 +23454,7 @@
       <c r="F178" s="20"/>
       <c r="G178" s="18"/>
     </row>
-    <row r="179" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" s="17" t="s">
         <v>73</v>
       </c>
@@ -23466,7 +23467,7 @@
       <c r="F179" s="20"/>
       <c r="G179" s="18"/>
     </row>
-    <row r="180" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" s="17" t="s">
         <v>634</v>
       </c>
@@ -23479,7 +23480,7 @@
       <c r="F180" s="20"/>
       <c r="G180" s="18"/>
     </row>
-    <row r="181" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" s="17" t="s">
         <v>75</v>
       </c>
@@ -23492,7 +23493,7 @@
       <c r="F181" s="20"/>
       <c r="G181" s="18"/>
     </row>
-    <row r="182" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" s="17" t="s">
         <v>77</v>
       </c>
@@ -23505,7 +23506,7 @@
       <c r="F182" s="20"/>
       <c r="G182" s="18"/>
     </row>
-    <row r="183" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" s="17" t="s">
         <v>79</v>
       </c>
@@ -23518,7 +23519,7 @@
       <c r="F183" s="20"/>
       <c r="G183" s="18"/>
     </row>
-    <row r="184" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184" s="17" t="s">
         <v>81</v>
       </c>
@@ -23531,7 +23532,7 @@
       <c r="F184" s="20"/>
       <c r="G184" s="18"/>
     </row>
-    <row r="185" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185" s="17" t="s">
         <v>83</v>
       </c>
@@ -23550,7 +23551,7 @@
       <c r="F185" s="20"/>
       <c r="G185" s="18"/>
     </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186" s="12" t="s">
         <v>83</v>
       </c>
@@ -23567,7 +23568,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A187" s="12" t="s">
         <v>83</v>
       </c>
@@ -23584,7 +23585,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188" s="12" t="s">
         <v>83</v>
       </c>
@@ -23601,7 +23602,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A189" s="12" t="s">
         <v>83</v>
       </c>
@@ -23618,7 +23619,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190" s="12" t="s">
         <v>83</v>
       </c>
@@ -23635,7 +23636,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191" s="12" t="s">
         <v>83</v>
       </c>
@@ -23655,7 +23656,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="192" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192" s="17" t="s">
         <v>85</v>
       </c>
@@ -23674,7 +23675,7 @@
       <c r="F192" s="20"/>
       <c r="G192" s="18"/>
     </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193" s="12" t="s">
         <v>85</v>
       </c>
@@ -23691,7 +23692,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A194" s="12" t="s">
         <v>85</v>
       </c>
@@ -23708,7 +23709,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A195" s="12" t="s">
         <v>85</v>
       </c>
@@ -23725,7 +23726,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196" s="12" t="s">
         <v>85</v>
       </c>
@@ -23742,7 +23743,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" s="12" t="s">
         <v>85</v>
       </c>
@@ -23759,7 +23760,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198" s="12" t="s">
         <v>85</v>
       </c>
@@ -23776,7 +23777,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="199" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" s="17" t="s">
         <v>87</v>
       </c>
@@ -23795,7 +23796,7 @@
       <c r="F199" s="20"/>
       <c r="G199" s="18"/>
     </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200" s="12" t="s">
         <v>87</v>
       </c>
@@ -23812,7 +23813,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A201" s="12" t="s">
         <v>87</v>
       </c>
@@ -23829,7 +23830,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="202" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A202" s="17" t="s">
         <v>647</v>
       </c>
@@ -23842,7 +23843,7 @@
       <c r="F202" s="20"/>
       <c r="G202" s="18"/>
     </row>
-    <row r="203" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A203" s="17" t="s">
         <v>648</v>
       </c>
@@ -23855,7 +23856,7 @@
       <c r="F203" s="20"/>
       <c r="G203" s="18"/>
     </row>
-    <row r="204" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A204" s="17" t="s">
         <v>649</v>
       </c>
@@ -23868,7 +23869,7 @@
       <c r="F204" s="20"/>
       <c r="G204" s="18"/>
     </row>
-    <row r="205" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A205" s="17" t="s">
         <v>650</v>
       </c>
@@ -23881,7 +23882,7 @@
       <c r="F205" s="20"/>
       <c r="G205" s="18"/>
     </row>
-    <row r="206" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A206" s="17" t="s">
         <v>89</v>
       </c>
@@ -23894,7 +23895,7 @@
       <c r="F206" s="20"/>
       <c r="G206" s="18"/>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207" s="12" t="s">
         <v>91</v>
       </c>
@@ -23911,7 +23912,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A208" s="12" t="s">
         <v>91</v>
       </c>
@@ -23928,7 +23929,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="209" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A209" s="12" t="s">
         <v>91</v>
       </c>
@@ -23945,7 +23946,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A210" s="12" t="s">
         <v>91</v>
       </c>
@@ -23962,7 +23963,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A211" s="12" t="s">
         <v>91</v>
       </c>
@@ -23979,7 +23980,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A212" s="12" t="s">
         <v>91</v>
       </c>
@@ -23996,7 +23997,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A213" s="12" t="s">
         <v>91</v>
       </c>
@@ -24013,7 +24014,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A214" s="12" t="s">
         <v>91</v>
       </c>
@@ -24030,7 +24031,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A215" s="12" t="s">
         <v>91</v>
       </c>
@@ -24047,7 +24048,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A216" s="12" t="s">
         <v>91</v>
       </c>
@@ -24064,7 +24065,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="217" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A217" s="17" t="s">
         <v>93</v>
       </c>
@@ -24083,7 +24084,7 @@
       <c r="F217" s="20"/>
       <c r="G217" s="18"/>
     </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A218" s="12" t="s">
         <v>93</v>
       </c>
@@ -24100,7 +24101,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A219" s="12" t="s">
         <v>93</v>
       </c>
@@ -24117,7 +24118,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A220" s="12" t="s">
         <v>93</v>
       </c>
@@ -24134,7 +24135,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A221" s="12" t="s">
         <v>93</v>
       </c>
@@ -24151,7 +24152,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A222" s="12" t="s">
         <v>93</v>
       </c>
@@ -24181,7 +24182,9 @@
       <c r="D223" s="39" t="s">
         <v>717</v>
       </c>
-      <c r="E223" s="17"/>
+      <c r="E223" s="39" t="s">
+        <v>717</v>
+      </c>
       <c r="F223" s="20"/>
       <c r="G223" s="18"/>
     </row>
@@ -24198,8 +24201,8 @@
       <c r="D224" s="40" t="s">
         <v>718</v>
       </c>
-      <c r="E224" s="12" t="s">
-        <v>717</v>
+      <c r="E224" s="40" t="s">
+        <v>718</v>
       </c>
     </row>
     <row r="225" spans="1:7" x14ac:dyDescent="0.25">
@@ -24215,8 +24218,8 @@
       <c r="D225" s="40" t="s">
         <v>719</v>
       </c>
-      <c r="E225" s="12" t="s">
-        <v>718</v>
+      <c r="E225" s="40" t="s">
+        <v>719</v>
       </c>
     </row>
     <row r="226" spans="1:7" x14ac:dyDescent="0.25">
@@ -24232,8 +24235,8 @@
       <c r="D226" s="40" t="s">
         <v>720</v>
       </c>
-      <c r="E226" s="12" t="s">
-        <v>719</v>
+      <c r="E226" s="40" t="s">
+        <v>720</v>
       </c>
     </row>
     <row r="227" spans="1:7" ht="45" x14ac:dyDescent="0.25">
@@ -24249,8 +24252,8 @@
       <c r="D227" s="40" t="s">
         <v>721</v>
       </c>
-      <c r="E227" s="12" t="s">
-        <v>720</v>
+      <c r="E227" s="40" t="s">
+        <v>721</v>
       </c>
     </row>
     <row r="228" spans="1:7" x14ac:dyDescent="0.25">
@@ -24266,11 +24269,11 @@
       <c r="D228" s="40" t="s">
         <v>730</v>
       </c>
-      <c r="E228" s="12" t="s">
-        <v>721</v>
-      </c>
-    </row>
-    <row r="229" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="E228" s="40" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="229" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A229" s="17" t="s">
         <v>95</v>
       </c>
@@ -24289,7 +24292,7 @@
       <c r="F229" s="20"/>
       <c r="G229" s="18"/>
     </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A230" s="12" t="s">
         <v>95</v>
       </c>
@@ -24306,7 +24309,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A231" s="12" t="s">
         <v>95</v>
       </c>
@@ -24323,7 +24326,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="232" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A232" s="17" t="s">
         <v>674</v>
       </c>
@@ -24342,7 +24345,7 @@
       <c r="F232" s="20"/>
       <c r="G232" s="18"/>
     </row>
-    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A233" s="12" t="s">
         <v>674</v>
       </c>
@@ -24359,7 +24362,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="234" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A234" s="17" t="s">
         <v>97</v>
       </c>
@@ -24378,7 +24381,7 @@
       <c r="F234" s="20"/>
       <c r="G234" s="18"/>
     </row>
-    <row r="235" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A235" s="12" t="s">
         <v>97</v>
       </c>
@@ -24395,7 +24398,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="236" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A236" s="12" t="s">
         <v>97</v>
       </c>
@@ -24412,7 +24415,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="237" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A237" s="17" t="s">
         <v>99</v>
       </c>
@@ -24431,7 +24434,7 @@
       <c r="F237" s="20"/>
       <c r="G237" s="18"/>
     </row>
-    <row r="238" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A238" s="12" t="s">
         <v>99</v>
       </c>
@@ -24448,7 +24451,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="239" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A239" s="12" t="s">
         <v>99</v>
       </c>
@@ -24465,7 +24468,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="240" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A240" s="17" t="s">
         <v>101</v>
       </c>
@@ -24484,7 +24487,7 @@
       <c r="F240" s="20"/>
       <c r="G240" s="18"/>
     </row>
-    <row r="241" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A241" s="12" t="s">
         <v>101</v>
       </c>
@@ -24501,7 +24504,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="242" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A242" s="12" t="s">
         <v>101</v>
       </c>
@@ -24518,7 +24521,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="243" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A243" s="17" t="s">
         <v>673</v>
       </c>
@@ -24531,7 +24534,7 @@
       <c r="F243" s="20"/>
       <c r="G243" s="18"/>
     </row>
-    <row r="244" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A244" s="17" t="s">
         <v>714</v>
       </c>
@@ -24550,7 +24553,7 @@
       <c r="F244" s="20"/>
       <c r="G244" s="18"/>
     </row>
-    <row r="245" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A245" s="12" t="s">
         <v>714</v>
       </c>
@@ -24567,7 +24570,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="246" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A246" s="17" t="s">
         <v>722</v>
       </c>
@@ -24586,7 +24589,7 @@
       <c r="F246" s="20"/>
       <c r="G246" s="18"/>
     </row>
-    <row r="247" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A247" s="12" t="s">
         <v>722</v>
       </c>
@@ -24603,7 +24606,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="248" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A248" s="12" t="s">
         <v>722</v>
       </c>
@@ -24620,7 +24623,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="249" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A249" s="12" t="s">
         <v>722</v>
       </c>
@@ -24637,7 +24640,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="250" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A250" s="12" t="s">
         <v>722</v>
       </c>
@@ -24654,7 +24657,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="251" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:7" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A251" s="12" t="s">
         <v>722</v>
       </c>
@@ -24671,7 +24674,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="252" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A252" s="12" t="s">
         <v>722</v>
       </c>
@@ -24688,7 +24691,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="253" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A253" s="17" t="s">
         <v>103</v>
       </c>
@@ -24707,7 +24710,7 @@
       <c r="F253" s="20"/>
       <c r="G253" s="18"/>
     </row>
-    <row r="254" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A254" s="12" t="s">
         <v>103</v>
       </c>
@@ -24724,7 +24727,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="255" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A255" s="12" t="s">
         <v>103</v>
       </c>
@@ -24741,7 +24744,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="256" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A256" s="17" t="s">
         <v>105</v>
       </c>
@@ -24760,7 +24763,7 @@
       <c r="F256" s="20"/>
       <c r="G256" s="18"/>
     </row>
-    <row r="257" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A257" s="12" t="s">
         <v>105</v>
       </c>
@@ -24777,7 +24780,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="258" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A258" s="12" t="s">
         <v>105</v>
       </c>
@@ -24794,7 +24797,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="259" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A259" s="17" t="s">
         <v>107</v>
       </c>
@@ -24813,7 +24816,7 @@
       <c r="F259" s="20"/>
       <c r="G259" s="18"/>
     </row>
-    <row r="260" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A260" s="12" t="s">
         <v>107</v>
       </c>
@@ -24830,7 +24833,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="261" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A261" s="12" t="s">
         <v>107</v>
       </c>
@@ -24847,7 +24850,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="262" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A262" s="17" t="s">
         <v>109</v>
       </c>
@@ -24866,7 +24869,7 @@
       <c r="F262" s="20"/>
       <c r="G262" s="18"/>
     </row>
-    <row r="263" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A263" s="12" t="s">
         <v>109</v>
       </c>
@@ -24883,7 +24886,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="264" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A264" s="12" t="s">
         <v>109</v>
       </c>
@@ -24900,7 +24903,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="265" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A265" s="17" t="s">
         <v>111</v>
       </c>
@@ -24919,7 +24922,7 @@
       <c r="F265" s="20"/>
       <c r="G265" s="18"/>
     </row>
-    <row r="266" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A266" s="12" t="s">
         <v>111</v>
       </c>
@@ -24936,7 +24939,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="267" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A267" s="12" t="s">
         <v>111</v>
       </c>
@@ -24953,7 +24956,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="268" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A268" s="17" t="s">
         <v>675</v>
       </c>
@@ -24972,7 +24975,7 @@
       <c r="F268" s="20"/>
       <c r="G268" s="18"/>
     </row>
-    <row r="269" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A269" s="12" t="s">
         <v>675</v>
       </c>
@@ -24989,7 +24992,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="270" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A270" s="17" t="s">
         <v>113</v>
       </c>
@@ -25008,7 +25011,7 @@
       <c r="F270" s="20"/>
       <c r="G270" s="18"/>
     </row>
-    <row r="271" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A271" s="12" t="s">
         <v>113</v>
       </c>
@@ -25025,7 +25028,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="272" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A272" s="12" t="s">
         <v>113</v>
       </c>
@@ -25042,7 +25045,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="273" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A273" s="17" t="s">
         <v>115</v>
       </c>
@@ -25061,7 +25064,7 @@
       <c r="F273" s="20"/>
       <c r="G273" s="18"/>
     </row>
-    <row r="274" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A274" s="12" t="s">
         <v>115</v>
       </c>
@@ -25078,7 +25081,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="275" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A275" s="12" t="s">
         <v>115</v>
       </c>
@@ -25095,7 +25098,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="276" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A276" s="17" t="s">
         <v>117</v>
       </c>
@@ -25114,7 +25117,7 @@
       <c r="F276" s="20"/>
       <c r="G276" s="18"/>
     </row>
-    <row r="277" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A277" s="12" t="s">
         <v>117</v>
       </c>
@@ -25131,7 +25134,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A278" s="12" t="s">
         <v>117</v>
       </c>
@@ -25148,7 +25151,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="279" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A279" s="17" t="s">
         <v>119</v>
       </c>
@@ -25167,7 +25170,7 @@
       <c r="F279" s="20"/>
       <c r="G279" s="18"/>
     </row>
-    <row r="280" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A280" s="12" t="s">
         <v>119</v>
       </c>
@@ -25184,7 +25187,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="281" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A281" s="12" t="s">
         <v>119</v>
       </c>
@@ -25201,7 +25204,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="282" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A282" s="17" t="s">
         <v>121</v>
       </c>
@@ -25220,7 +25223,7 @@
       <c r="F282" s="20"/>
       <c r="G282" s="18"/>
     </row>
-    <row r="283" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A283" s="12" t="s">
         <v>121</v>
       </c>
@@ -25237,7 +25240,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="284" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A284" s="12" t="s">
         <v>121</v>
       </c>
@@ -25254,7 +25257,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="285" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A285" s="12" t="s">
         <v>121</v>
       </c>
@@ -25271,7 +25274,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="286" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A286" s="12" t="s">
         <v>121</v>
       </c>
@@ -25288,7 +25291,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="287" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A287" s="12" t="s">
         <v>121</v>
       </c>
@@ -25305,7 +25308,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="288" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A288" s="12" t="s">
         <v>121</v>
       </c>
@@ -25322,7 +25325,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A289" s="12" t="s">
         <v>121</v>
       </c>
@@ -25339,7 +25342,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A290" s="12" t="s">
         <v>121</v>
       </c>
@@ -25356,7 +25359,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A291" s="12" t="s">
         <v>121</v>
       </c>
@@ -25373,7 +25376,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A292" s="12" t="s">
         <v>121</v>
       </c>
@@ -25390,7 +25393,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A293" s="12" t="s">
         <v>121</v>
       </c>
@@ -25407,7 +25410,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A294" s="12" t="s">
         <v>121</v>
       </c>
@@ -25424,7 +25427,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A295" s="12" t="s">
         <v>121</v>
       </c>
@@ -25441,7 +25444,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A296" s="12" t="s">
         <v>121</v>
       </c>
@@ -25458,7 +25461,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A297" s="12" t="s">
         <v>121</v>
       </c>
@@ -25475,7 +25478,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A298" s="12" t="s">
         <v>121</v>
       </c>
@@ -25492,7 +25495,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A299" s="12" t="s">
         <v>121</v>
       </c>
@@ -25509,7 +25512,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A300" s="12" t="s">
         <v>121</v>
       </c>
@@ -25526,7 +25529,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="301" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:5" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A301" s="12" t="s">
         <v>121</v>
       </c>
@@ -25543,7 +25546,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A302" s="12" t="s">
         <v>121</v>
       </c>
@@ -25560,7 +25563,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A303" s="12" t="s">
         <v>121</v>
       </c>
@@ -25577,7 +25580,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="304" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:5" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A304" s="12" t="s">
         <v>121</v>
       </c>
@@ -25594,7 +25597,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="305" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A305" s="12" t="s">
         <v>121</v>
       </c>
@@ -25611,7 +25614,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="306" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A306" s="12" t="s">
         <v>121</v>
       </c>
@@ -25628,7 +25631,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="307" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A307" s="12" t="s">
         <v>121</v>
       </c>
@@ -25645,7 +25648,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="308" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A308" s="12" t="s">
         <v>121</v>
       </c>
@@ -25662,7 +25665,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="309" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A309" s="12" t="s">
         <v>121</v>
       </c>
@@ -25679,7 +25682,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="310" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A310" s="12" t="s">
         <v>121</v>
       </c>
@@ -25696,7 +25699,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="311" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A311" s="12" t="s">
         <v>121</v>
       </c>
@@ -25713,7 +25716,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="312" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A312" s="12" t="s">
         <v>121</v>
       </c>
@@ -25730,7 +25733,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="313" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A313" s="12" t="s">
         <v>121</v>
       </c>
@@ -25747,7 +25750,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="314" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A314" s="19" t="s">
         <v>123</v>
       </c>
@@ -25766,7 +25769,7 @@
       <c r="F314" s="20"/>
       <c r="G314" s="18"/>
     </row>
-    <row r="315" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A315" s="4" t="s">
         <v>123</v>
       </c>
@@ -25783,7 +25786,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="316" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A316" s="4" t="s">
         <v>123</v>
       </c>
@@ -25800,7 +25803,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="317" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A317" s="19" t="s">
         <v>125</v>
       </c>
@@ -25819,7 +25822,7 @@
       <c r="F317" s="20"/>
       <c r="G317" s="18"/>
     </row>
-    <row r="318" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A318" s="4" t="s">
         <v>125</v>
       </c>
@@ -25836,7 +25839,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="319" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A319" s="4" t="s">
         <v>125</v>
       </c>
@@ -25853,7 +25856,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="320" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A320" s="19" t="s">
         <v>127</v>
       </c>
@@ -25866,7 +25869,7 @@
       <c r="F320" s="20"/>
       <c r="G320" s="18"/>
     </row>
-    <row r="321" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A321" s="19" t="s">
         <v>149</v>
       </c>
@@ -25879,7 +25882,7 @@
       <c r="F321" s="20"/>
       <c r="G321" s="18"/>
     </row>
-    <row r="322" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A322" s="19" t="s">
         <v>153</v>
       </c>
@@ -25892,7 +25895,7 @@
       <c r="F322" s="20"/>
       <c r="G322" s="18"/>
     </row>
-    <row r="323" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A323" s="19" t="s">
         <v>155</v>
       </c>
@@ -25905,7 +25908,7 @@
       <c r="F323" s="20"/>
       <c r="G323" s="18"/>
     </row>
-    <row r="324" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A324" s="19" t="s">
         <v>157</v>
       </c>
@@ -25918,7 +25921,7 @@
       <c r="F324" s="20"/>
       <c r="G324" s="18"/>
     </row>
-    <row r="325" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A325" s="19" t="s">
         <v>159</v>
       </c>
@@ -25931,7 +25934,7 @@
       <c r="F325" s="20"/>
       <c r="G325" s="18"/>
     </row>
-    <row r="326" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A326" s="19" t="s">
         <v>161</v>
       </c>
@@ -25944,7 +25947,7 @@
       <c r="F326" s="20"/>
       <c r="G326" s="18"/>
     </row>
-    <row r="327" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A327" s="19" t="s">
         <v>163</v>
       </c>
@@ -25957,7 +25960,7 @@
       <c r="F327" s="20"/>
       <c r="G327" s="18"/>
     </row>
-    <row r="328" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A328" s="19" t="s">
         <v>165</v>
       </c>
@@ -25970,7 +25973,7 @@
       <c r="F328" s="20"/>
       <c r="G328" s="18"/>
     </row>
-    <row r="329" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A329" s="19" t="s">
         <v>129</v>
       </c>
@@ -25983,7 +25986,7 @@
       <c r="F329" s="20"/>
       <c r="G329" s="18"/>
     </row>
-    <row r="330" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A330" s="19" t="s">
         <v>131</v>
       </c>
@@ -25996,7 +25999,7 @@
       <c r="F330" s="20"/>
       <c r="G330" s="18"/>
     </row>
-    <row r="331" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A331" s="19" t="s">
         <v>133</v>
       </c>
@@ -26009,7 +26012,7 @@
       <c r="F331" s="20"/>
       <c r="G331" s="18"/>
     </row>
-    <row r="332" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A332" s="19" t="s">
         <v>135</v>
       </c>
@@ -26022,7 +26025,7 @@
       <c r="F332" s="20"/>
       <c r="G332" s="18"/>
     </row>
-    <row r="333" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A333" s="19" t="s">
         <v>137</v>
       </c>
@@ -26035,7 +26038,7 @@
       <c r="F333" s="20"/>
       <c r="G333" s="18"/>
     </row>
-    <row r="334" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A334" s="19" t="s">
         <v>139</v>
       </c>
@@ -26048,7 +26051,7 @@
       <c r="F334" s="20"/>
       <c r="G334" s="18"/>
     </row>
-    <row r="335" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A335" s="19" t="s">
         <v>141</v>
       </c>
@@ -26061,7 +26064,7 @@
       <c r="F335" s="20"/>
       <c r="G335" s="18"/>
     </row>
-    <row r="336" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A336" s="19" t="s">
         <v>143</v>
       </c>
@@ -26074,7 +26077,7 @@
       <c r="F336" s="20"/>
       <c r="G336" s="18"/>
     </row>
-    <row r="337" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A337" s="19" t="s">
         <v>145</v>
       </c>
@@ -26087,7 +26090,7 @@
       <c r="F337" s="20"/>
       <c r="G337" s="18"/>
     </row>
-    <row r="338" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A338" s="19" t="s">
         <v>147</v>
       </c>
@@ -26100,7 +26103,7 @@
       <c r="F338" s="20"/>
       <c r="G338" s="18"/>
     </row>
-    <row r="339" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A339" s="19" t="s">
         <v>151</v>
       </c>
@@ -26113,7 +26116,7 @@
       <c r="F339" s="20"/>
       <c r="G339" s="18"/>
     </row>
-    <row r="340" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A340" s="17" t="s">
         <v>167</v>
       </c>
@@ -26132,7 +26135,7 @@
       <c r="F340" s="20"/>
       <c r="G340" s="18"/>
     </row>
-    <row r="341" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A341" s="12" t="s">
         <v>167</v>
       </c>
@@ -26149,7 +26152,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="342" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A342" s="12" t="s">
         <v>167</v>
       </c>
@@ -26166,7 +26169,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="343" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A343" s="19" t="s">
         <v>168</v>
       </c>
@@ -26179,7 +26182,7 @@
       <c r="F343" s="20"/>
       <c r="G343" s="18"/>
     </row>
-    <row r="344" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A344" s="19" t="s">
         <v>169</v>
       </c>
@@ -26192,7 +26195,7 @@
       <c r="F344" s="20"/>
       <c r="G344" s="18"/>
     </row>
-    <row r="345" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A345" s="19" t="s">
         <v>170</v>
       </c>
@@ -26205,7 +26208,7 @@
       <c r="F345" s="20"/>
       <c r="G345" s="18"/>
     </row>
-    <row r="346" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A346" s="19" t="s">
         <v>172</v>
       </c>
@@ -26218,7 +26221,7 @@
       <c r="F346" s="20"/>
       <c r="G346" s="18"/>
     </row>
-    <row r="347" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A347" s="19" t="s">
         <v>174</v>
       </c>
@@ -26231,7 +26234,7 @@
       <c r="F347" s="20"/>
       <c r="G347" s="18"/>
     </row>
-    <row r="348" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A348" s="19" t="s">
         <v>176</v>
       </c>
@@ -26244,7 +26247,7 @@
       <c r="F348" s="20"/>
       <c r="G348" s="18"/>
     </row>
-    <row r="349" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A349" s="17" t="s">
         <v>178</v>
       </c>
@@ -26263,7 +26266,7 @@
       <c r="F349" s="20"/>
       <c r="G349" s="18"/>
     </row>
-    <row r="350" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A350" s="12" t="s">
         <v>178</v>
       </c>
@@ -26280,7 +26283,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="351" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A351" s="12" t="s">
         <v>178</v>
       </c>
@@ -26297,7 +26300,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="352" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A352" s="12" t="s">
         <v>178</v>
       </c>
@@ -26314,7 +26317,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="353" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A353" s="12" t="s">
         <v>178</v>
       </c>
@@ -26331,7 +26334,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="354" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A354" s="12" t="s">
         <v>178</v>
       </c>
@@ -26348,7 +26351,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="355" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A355" s="12" t="s">
         <v>178</v>
       </c>
@@ -26365,7 +26368,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="356" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A356" s="17" t="s">
         <v>180</v>
       </c>
@@ -26378,7 +26381,7 @@
       <c r="F356" s="20"/>
       <c r="G356" s="18"/>
     </row>
-    <row r="357" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A357" s="17" t="s">
         <v>182</v>
       </c>
@@ -26391,7 +26394,7 @@
       <c r="F357" s="20"/>
       <c r="G357" s="18"/>
     </row>
-    <row r="358" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A358" s="19" t="s">
         <v>183</v>
       </c>
@@ -26410,7 +26413,7 @@
       <c r="F358" s="20"/>
       <c r="G358" s="18"/>
     </row>
-    <row r="359" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A359" s="4" t="s">
         <v>183</v>
       </c>
@@ -26427,7 +26430,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="360" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A360" s="4" t="s">
         <v>183</v>
       </c>
@@ -26444,7 +26447,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="361" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A361" s="4" t="s">
         <v>183</v>
       </c>
@@ -26464,7 +26467,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="362" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A362" s="19" t="s">
         <v>651</v>
       </c>
@@ -26476,7 +26479,7 @@
       <c r="E362" s="19"/>
       <c r="F362" s="20"/>
     </row>
-    <row r="363" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A363" s="19" t="s">
         <v>527</v>
       </c>
@@ -26489,7 +26492,7 @@
       <c r="F363" s="20"/>
       <c r="G363" s="18"/>
     </row>
-    <row r="364" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A364" s="19" t="s">
         <v>185</v>
       </c>
@@ -26502,7 +26505,7 @@
       <c r="F364" s="20"/>
       <c r="G364" s="18"/>
     </row>
-    <row r="365" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A365" s="19" t="s">
         <v>186</v>
       </c>
@@ -26515,7 +26518,7 @@
       <c r="F365" s="20"/>
       <c r="G365" s="18"/>
     </row>
-    <row r="366" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A366" s="19" t="s">
         <v>191</v>
       </c>
@@ -26528,7 +26531,7 @@
       <c r="F366" s="20"/>
       <c r="G366" s="18"/>
     </row>
-    <row r="367" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A367" s="17" t="s">
         <v>197</v>
       </c>
@@ -26547,7 +26550,7 @@
       <c r="F367" s="20"/>
       <c r="G367" s="18"/>
     </row>
-    <row r="368" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A368" s="12" t="s">
         <v>197</v>
       </c>
@@ -26564,7 +26567,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="369" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A369" s="12" t="s">
         <v>197</v>
       </c>
@@ -26581,7 +26584,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="370" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A370" s="12" t="s">
         <v>197</v>
       </c>
@@ -26598,7 +26601,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="371" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A371" s="19" t="s">
         <v>199</v>
       </c>
@@ -26611,7 +26614,7 @@
       <c r="F371" s="20"/>
       <c r="G371" s="18"/>
     </row>
-    <row r="372" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:7" s="21" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A372" s="19" t="s">
         <v>529</v>
       </c>
@@ -26625,7 +26628,13 @@
       <c r="G372" s="18"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G372" xr:uid="{51D60DD1-DC0B-4658-A996-7DC0B41964ED}"/>
+  <autoFilter ref="A1:G372" xr:uid="{51D60DD1-DC0B-4658-A996-7DC0B41964ED}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="race6"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>